<commit_message>
Actualiza portafolio 2026-06-22 17:50 UTC
</commit_message>
<xml_diff>
--- a/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
+++ b/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
@@ -4350,7 +4350,7 @@
       </c>
       <c r="C41" s="9"/>
       <c r="D41" s="8">
-        <v>46182.678233125</v>
+        <v>46195.71615581018</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>149</v>
@@ -4541,7 +4541,7 @@
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46195.68193791667</v>
+        <v>46195.71674362269</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>158</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-06-23 15:57 UTC
</commit_message>
<xml_diff>
--- a/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
+++ b/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
@@ -3535,7 +3535,7 @@
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="5">
-        <v>46193.20103372685</v>
+        <v>46196.65421123843</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>105</v>
@@ -3580,13 +3580,13 @@
         <v>46192</v>
       </c>
       <c r="S28" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T28" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U28" s="12" t="s">
-        <v>90</v>
+      <c r="U28" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="5">
-        <v>46195.714815196756</v>
+        <v>46196.634982337964</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>134</v>
@@ -4732,7 +4732,7 @@
       </c>
       <c r="C47" s="9"/>
       <c r="D47" s="8">
-        <v>46169.856877048616</v>
+        <v>46196.654216180556</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>109</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-07-07 11:15 Chile
</commit_message>
<xml_diff>
--- a/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
+++ b/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
@@ -3538,7 +3538,7 @@
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="5">
-        <v>46210.57522067129</v>
+        <v>46210.62912240741</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>105</v>
@@ -3583,7 +3583,7 @@
         <v>46192</v>
       </c>
       <c r="S28" s="6">
-        <v>1</v>
+        <v>0.66</v>
       </c>
       <c r="T28" s="10" t="s">
         <v>31</v>
@@ -3666,7 +3666,7 @@
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="5">
-        <v>46209.586068969904</v>
+        <v>46210.62940358796</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>114</v>
@@ -3711,7 +3711,7 @@
         <v>46192</v>
       </c>
       <c r="S30" s="6">
-        <v>0</v>
+        <v>0.66</v>
       </c>
       <c r="T30" s="10" t="s">
         <v>31</v>
@@ -3731,7 +3731,7 @@
         <v>46113.808467152776</v>
       </c>
       <c r="D31" s="8">
-        <v>46123.18662818287</v>
+        <v>46210.62933210648</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>86</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-07-07 12:37 Chile
</commit_message>
<xml_diff>
--- a/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
+++ b/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
@@ -250,7 +250,7 @@
     <t>Ingenieria Detalle</t>
   </si>
   <si>
-    <t>Ingenieria Jefe de proyecto:,Propuesta Sensores,Analisis de costeo,Propuesta Fabricacion Externa  ot 4294 - 4296 - 4297,Planos preliminar,OT 4294 ZVR 1-14-42/4,OT 4296 ZVR 1-14-34/4,OT 4297 ZVR1-14-25/4</t>
+    <t>Ingenieria Jefe de proyecto:,Propuesta Sensores,Analisis de costeo,Propuesta Fabricación Externa  ot 4294 - 4296 - 4297,Planos preliminar,OT 4294 ZVR 1-14-42/4,OT 4296 ZVR 1-14-34/4,OT 4297 ZVR1-14-25/4</t>
   </si>
   <si>
     <t>1213886181447052</t>
@@ -355,7 +355,7 @@
     <t>1213886181474407</t>
   </si>
   <si>
-    <t>Propuesta Fabricacion Externa  ot 4294 - 4296 - 4297</t>
+    <t>Propuesta Fabricación Externa  ot 4294 - 4296 - 4297</t>
   </si>
   <si>
     <t>Ingenieria Detalle,Check Planos</t>
@@ -721,7 +721,7 @@
     <t>1213886181537550</t>
   </si>
   <si>
-    <t>Fabricacion Externa  ot 4294 - 4296 - 4297,Fabricacion estructura proveedor externo  ot 4294 - 4296 - 4297,OT 4296 ZVR1-14-34/4,OT 4296 ZVR1-14-34/4,OT 4294 ZVR 1-14-42/4,OT 4294 ZVR 1-14-42/4,OT 4294 ZVR 1-14-42/4,OT 4294 ZVR 1-14-42/4,OT 4296 ZVR1-14-34/4,OT 4294 ZVR 1-14-42/4,OT 4294 ZVR 1-14-42/4,OT 4296 ZVR1-14-34/4,OT 4296 ZVR1-14-34/4,OT 4296 ZVR1-14-34/4,propuesta compras a codigo // aprovisionamiento ot 4294 - 4296 - 4297,Propuesta Fabricacion Externa  ot 4294 - 4296 - 4297</t>
+    <t>Fabricacion Externa  ot 4294 - 4296 - 4297,Fabricacion estructura proveedor externo  ot 4294 - 4296 - 4297,OT 4296 ZVR1-14-34/4,OT 4296 ZVR1-14-34/4,OT 4294 ZVR 1-14-42/4,OT 4294 ZVR 1-14-42/4,OT 4294 ZVR 1-14-42/4,OT 4294 ZVR 1-14-42/4,OT 4296 ZVR1-14-34/4,OT 4294 ZVR 1-14-42/4,OT 4294 ZVR 1-14-42/4,OT 4296 ZVR1-14-34/4,OT 4296 ZVR1-14-34/4,OT 4296 ZVR1-14-34/4,propuesta compras a codigo // aprovisionamiento ot 4294 - 4296 - 4297,Propuesta Fabricación Externa  ot 4294 - 4296 - 4297</t>
   </si>
   <si>
     <t>1213910573903658</t>
@@ -3666,7 +3666,7 @@
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="5">
-        <v>46210.62940358796</v>
+        <v>46210.672841631946</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>114</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-03 20:43 UTC
</commit_message>
<xml_diff>
--- a/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
+++ b/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
@@ -6470,7 +6470,7 @@
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46114.74446109954</v>
+        <v>46237.84762954861</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>261</v>
@@ -6578,9 +6578,11 @@
       <c r="B79" s="8">
         <v>46112.679890740736</v>
       </c>
-      <c r="C79" s="9"/>
+      <c r="C79" s="8">
+        <v>46237.84762318287</v>
+      </c>
       <c r="D79" s="8">
-        <v>46179.167811527775</v>
+        <v>46237.847639803236</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>269</v>
@@ -6625,13 +6627,13 @@
         <v>46178</v>
       </c>
       <c r="S79" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T79" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U79" s="10" t="s">
-        <v>54</v>
+      <c r="U79" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
@@ -6690,7 +6692,7 @@
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46226.20781865741</v>
+        <v>46237.847639803236</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>275</v>
@@ -6740,8 +6742,8 @@
       <c r="T81" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U81" s="10" t="s">
-        <v>54</v>
+      <c r="U81" s="12" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-08-03 21:18 UTC
</commit_message>
<xml_diff>
--- a/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
+++ b/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1983" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1984" uniqueCount="486">
   <si>
     <t>50001534-ZITRON PERU METRO DE LIMA (E04-05 06-R4)</t>
   </si>
@@ -586,7 +586,7 @@
     <t>Generacion OC Fabricacion Externa  ot 4294 - 4296 - 4297,Fabricacion a codigo y compras locales ot 4294 - 4296 - 4297,Check Planos,Planos preliminar</t>
   </si>
   <si>
-    <t>Fabricacion Externa  ot 4294 - 4296 - 4297,Control de calidad Fabricación externa</t>
+    <t>Fabricacion Externa  ot 4294 - 4296 - 4297,Control de calidad Fabricación externa  4294 - 4296 - 4297</t>
   </si>
   <si>
     <t>1213886259324444</t>
@@ -775,7 +775,7 @@
     <t>Control de calidad</t>
   </si>
   <si>
-    <t>Control de calidad Fabricación externa</t>
+    <t>Control de calidad Fabricación externa  4294 - 4296 - 4297</t>
   </si>
   <si>
     <t>1213902113480444</t>
@@ -6409,7 +6409,7 @@
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46232.188831238425</v>
+        <v>46237.86113535879</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>254</v>
@@ -6468,9 +6468,11 @@
       <c r="B77" s="8">
         <v>46112.6798790162</v>
       </c>
-      <c r="C77" s="9"/>
+      <c r="C77" s="8">
+        <v>46237.86031974537</v>
+      </c>
       <c r="D77" s="8">
-        <v>46237.84762954861</v>
+        <v>46237.86033361111</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>261</v>
@@ -6504,9 +6506,13 @@
       </c>
       <c r="Q77" s="9"/>
       <c r="R77" s="9"/>
-      <c r="S77" s="9"/>
+      <c r="S77" s="9">
+        <v>1</v>
+      </c>
       <c r="T77" s="9"/>
-      <c r="U77" s="9"/>
+      <c r="U77" s="11" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
@@ -6515,9 +6521,11 @@
       <c r="B78" s="5">
         <v>46112.6798825463</v>
       </c>
-      <c r="C78" s="6"/>
+      <c r="C78" s="5">
+        <v>46237.86030320602</v>
+      </c>
       <c r="D78" s="5">
-        <v>46211.830947395836</v>
+        <v>46237.86031981482</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>264</v>
@@ -6562,13 +6570,13 @@
         <v>46176</v>
       </c>
       <c r="S78" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T78" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U78" s="12" t="s">
-        <v>259</v>
+      <c r="U78" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
@@ -6582,7 +6590,7 @@
         <v>46237.84762318287</v>
       </c>
       <c r="D79" s="8">
-        <v>46237.847639803236</v>
+        <v>46237.86032310185</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>269</v>
@@ -6632,8 +6640,8 @@
       <c r="T79" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U79" s="11" t="s">
-        <v>32</v>
+      <c r="U79" s="12" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-08-26 20:17 UTC
</commit_message>
<xml_diff>
--- a/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
+++ b/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1947" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1948" uniqueCount="478">
   <si>
     <t>50001534-ZITRON PERU METRO DE LIMA (E04-05 06-R4)</t>
   </si>
@@ -787,40 +787,40 @@
     <t>Control de calidad,Recepcion Fabricacion externa</t>
   </si>
   <si>
+    <t>1213902113485641</t>
+  </si>
+  <si>
+    <t>Bodega</t>
+  </si>
+  <si>
+    <t>Recepcion materiales a codigos // compras locales aprovisionamiento,Control de calidad compras materiales a codigo // compras locale aprovisionamient</t>
+  </si>
+  <si>
+    <t>1213886181542206</t>
+  </si>
+  <si>
+    <t>Recepcion materiales a codigos // compras locales aprovisionamiento</t>
+  </si>
+  <si>
+    <t>Victor Muñoz</t>
+  </si>
+  <si>
+    <t>victor.munoz@zitron.com</t>
+  </si>
+  <si>
+    <t>Bodega,Control de calidad compras materiales a codigo // compras locale aprovisionamient</t>
+  </si>
+  <si>
+    <t>1213886181542236</t>
+  </si>
+  <si>
+    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamient</t>
+  </si>
+  <si>
+    <t>Bodega,Preparacion materiales</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1213902113485641</t>
-  </si>
-  <si>
-    <t>Bodega</t>
-  </si>
-  <si>
-    <t>Recepcion materiales a codigos // compras locales aprovisionamiento,Control de calidad compras materiales a codigo // compras locale aprovisionamient</t>
-  </si>
-  <si>
-    <t>1213886181542206</t>
-  </si>
-  <si>
-    <t>Recepcion materiales a codigos // compras locales aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Victor Muñoz</t>
-  </si>
-  <si>
-    <t>victor.munoz@zitron.com</t>
-  </si>
-  <si>
-    <t>Bodega,Control de calidad compras materiales a codigo // compras locale aprovisionamient</t>
-  </si>
-  <si>
-    <t>1213886181542236</t>
-  </si>
-  <si>
-    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamient</t>
-  </si>
-  <si>
-    <t>Bodega,Preparacion materiales</t>
   </si>
   <si>
     <t>1213902113596084</t>
@@ -6336,9 +6336,11 @@
       <c r="B75" s="8">
         <v>46112.679867326384</v>
       </c>
-      <c r="C75" s="9"/>
+      <c r="C75" s="8">
+        <v>46260.658577766204</v>
+      </c>
       <c r="D75" s="8">
-        <v>46118.55096414352</v>
+        <v>46260.658590023144</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>252</v>
@@ -6372,9 +6374,13 @@
       </c>
       <c r="Q75" s="9"/>
       <c r="R75" s="9"/>
-      <c r="S75" s="9"/>
+      <c r="S75" s="9">
+        <v>1</v>
+      </c>
       <c r="T75" s="9"/>
-      <c r="U75" s="9"/>
+      <c r="U75" s="11" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
@@ -6383,9 +6389,11 @@
       <c r="B76" s="5">
         <v>46112.67987047454</v>
       </c>
-      <c r="C76" s="6"/>
+      <c r="C76" s="5">
+        <v>46260.65855825231</v>
+      </c>
       <c r="D76" s="5">
-        <v>46239.167648125</v>
+        <v>46260.65857824074</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>253</v>
@@ -6428,18 +6436,18 @@
         <v>46231</v>
       </c>
       <c r="S76" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T76" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U76" s="12" t="s">
-        <v>258</v>
+      <c r="U76" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B77" s="8">
         <v>46112.6798790162</v>
@@ -6451,7 +6459,7 @@
         <v>46237.86033361111</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>25</v>
@@ -6475,7 +6483,7 @@
         <v>26</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="P77" s="9" t="s">
         <v>26</v>
@@ -6492,7 +6500,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B78" s="5">
         <v>46112.6798825463</v>
@@ -6504,16 +6512,16 @@
         <v>46237.86031981482</v>
       </c>
       <c r="E78" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G78" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="F78" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G78" s="6" t="s">
+      <c r="H78" s="6" t="s">
         <v>264</v>
-      </c>
-      <c r="H78" s="6" t="s">
-        <v>265</v>
       </c>
       <c r="I78" s="5">
         <v>46244</v>
@@ -6531,13 +6539,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="O78" s="6" t="s">
         <v>169</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="Q78" s="5">
         <v>46175</v>
@@ -6557,7 +6565,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B79" s="8">
         <v>46112.679890740736</v>
@@ -6569,7 +6577,7 @@
         <v>46237.86032310185</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>26</v>
@@ -6596,13 +6604,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="Q79" s="8">
         <v>46177</v>
@@ -6617,7 +6625,7 @@
         <v>31</v>
       </c>
       <c r="U79" s="12" t="s">
-        <v>258</v>
+        <v>269</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
@@ -6711,7 +6719,7 @@
         <v>271</v>
       </c>
       <c r="O81" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="P81" s="9" t="s">
         <v>277</v>
@@ -6741,7 +6749,7 @@
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46260.583539328705</v>
+        <v>46260.65928364583</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>279</v>
@@ -7245,10 +7253,10 @@
         <v>26</v>
       </c>
       <c r="G91" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="H91" s="9" t="s">
         <v>264</v>
-      </c>
-      <c r="H91" s="9" t="s">
-        <v>265</v>
       </c>
       <c r="I91" s="8">
         <v>46183</v>
@@ -7308,10 +7316,10 @@
         <v>26</v>
       </c>
       <c r="G92" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="H92" s="6" t="s">
         <v>264</v>
-      </c>
-      <c r="H92" s="6" t="s">
-        <v>265</v>
       </c>
       <c r="I92" s="5">
         <v>46239</v>
@@ -7371,10 +7379,10 @@
         <v>26</v>
       </c>
       <c r="G93" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="H93" s="9" t="s">
         <v>264</v>
-      </c>
-      <c r="H93" s="9" t="s">
-        <v>265</v>
       </c>
       <c r="I93" s="8">
         <v>46246</v>
@@ -7413,7 +7421,7 @@
         <v>31</v>
       </c>
       <c r="U93" s="12" t="s">
-        <v>258</v>
+        <v>269</v>
       </c>
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
@@ -7434,10 +7442,10 @@
         <v>26</v>
       </c>
       <c r="G94" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="H94" s="6" t="s">
         <v>264</v>
-      </c>
-      <c r="H94" s="6" t="s">
-        <v>265</v>
       </c>
       <c r="I94" s="5">
         <v>46273</v>
@@ -7497,10 +7505,10 @@
         <v>26</v>
       </c>
       <c r="G95" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="H95" s="9" t="s">
         <v>264</v>
-      </c>
-      <c r="H95" s="9" t="s">
-        <v>265</v>
       </c>
       <c r="I95" s="8">
         <v>46220</v>
@@ -7539,7 +7547,7 @@
         <v>31</v>
       </c>
       <c r="U95" s="12" t="s">
-        <v>258</v>
+        <v>269</v>
       </c>
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
@@ -7551,7 +7559,7 @@
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46239.16765043982</v>
+        <v>46260.6585802662</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>316</v>
@@ -7560,10 +7568,10 @@
         <v>26</v>
       </c>
       <c r="G96" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="H96" s="6" t="s">
         <v>264</v>
-      </c>
-      <c r="H96" s="6" t="s">
-        <v>265</v>
       </c>
       <c r="I96" s="6"/>
       <c r="J96" s="5">
@@ -7599,8 +7607,8 @@
       <c r="T96" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U96" s="10" t="s">
-        <v>53</v>
+      <c r="U96" s="12" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
@@ -7621,10 +7629,10 @@
         <v>26</v>
       </c>
       <c r="G97" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="H97" s="9" t="s">
         <v>264</v>
-      </c>
-      <c r="H97" s="9" t="s">
-        <v>265</v>
       </c>
       <c r="I97" s="8">
         <v>46181</v>
@@ -7663,7 +7671,7 @@
         <v>31</v>
       </c>
       <c r="U97" s="12" t="s">
-        <v>258</v>
+        <v>269</v>
       </c>
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizacion automatica 2026-08-31 23:54 UTC
</commit_message>
<xml_diff>
--- a/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
+++ b/data/50001534 - ZITRON PERU METRO LIMA E04-05-06-R4.xlsx
@@ -6637,7 +6637,7 @@
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46260.58241461805</v>
+        <v>46265.8665325926</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>272</v>
@@ -6973,9 +6973,11 @@
       <c r="B86" s="5">
         <v>46112.6799821875</v>
       </c>
-      <c r="C86" s="6"/>
+      <c r="C86" s="5">
+        <v>46265.866524791665</v>
+      </c>
       <c r="D86" s="5">
-        <v>46255.5535544213</v>
+        <v>46265.866544212964</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>289</v>
@@ -7020,13 +7022,13 @@
         <v>46247</v>
       </c>
       <c r="S86" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T86" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U86" s="10" t="s">
-        <v>53</v>
+      <c r="U86" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>